<commit_message>
feat(auditor): actualización de reglas de validación y firma de autor
</commit_message>
<xml_diff>
--- a/SEG FEB 2026FOMAG.xlsx
+++ b/SEG FEB 2026FOMAG.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Registro_datos_excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\aplicaciones hsv\Registro_datos_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A93B4E5-8361-4871-8ED5-CAF9BDD28C04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F088BEFE-B248-4B23-8CC1-B473BA778B48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="25440" windowHeight="15270" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35010,7 +35010,7 @@
     <col min="4" max="4" width="16.5546875" customWidth="1"/>
     <col min="5" max="5" width="24.109375" customWidth="1"/>
     <col min="6" max="6" width="18.44140625" customWidth="1"/>
-    <col min="7" max="7" width="12.6640625" customWidth="1"/>
+    <col min="7" max="7" width="26.88671875" customWidth="1"/>
     <col min="8" max="8" width="38.109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -35051,19 +35051,19 @@
         <v>239</v>
       </c>
       <c r="D2" s="12">
-        <v>1928261</v>
+        <v>1912678</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>247</v>
+        <v>287</v>
       </c>
       <c r="F2" s="13">
-        <v>46054.381184259255</v>
+        <v>46062.791729201388</v>
       </c>
       <c r="G2" s="12">
-        <v>1076900</v>
+        <v>71500</v>
       </c>
       <c r="H2" s="12" t="s">
-        <v>267</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -35077,19 +35077,19 @@
         <v>239</v>
       </c>
       <c r="D3" s="12">
-        <v>1911983</v>
+        <v>1931867</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>297</v>
+        <v>1837</v>
       </c>
       <c r="F3" s="13">
-        <v>46055.423922141199</v>
+        <v>46065.541980787035</v>
       </c>
       <c r="G3" s="12">
-        <v>902600</v>
+        <v>75000</v>
       </c>
       <c r="H3" s="12" t="s">
-        <v>65</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
@@ -35138,7 +35138,7 @@
         <v>46059.367089930551</v>
       </c>
       <c r="G5" s="12">
-        <v>79100</v>
+        <v>50001000</v>
       </c>
       <c r="H5" s="12" t="s">
         <v>27</v>
@@ -35207,19 +35207,19 @@
         <v>239</v>
       </c>
       <c r="D8" s="12">
-        <v>1912678</v>
+        <v>1931413</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>287</v>
+        <v>1839</v>
       </c>
       <c r="F8" s="13">
-        <v>46062.791729201388</v>
+        <v>46064.372635300926</v>
       </c>
       <c r="G8" s="12">
-        <v>71500</v>
+        <v>79100</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>65</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
@@ -35233,19 +35233,19 @@
         <v>239</v>
       </c>
       <c r="D9" s="12">
-        <v>1931413</v>
+        <v>1911983</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>1839</v>
+        <v>297</v>
       </c>
       <c r="F9" s="13">
-        <v>46064.372635300926</v>
+        <v>46055.423922141199</v>
       </c>
       <c r="G9" s="12">
-        <v>79100</v>
+        <v>902600</v>
       </c>
       <c r="H9" s="12" t="s">
-        <v>27</v>
+        <v>65</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
@@ -35259,19 +35259,19 @@
         <v>239</v>
       </c>
       <c r="D10" s="12">
-        <v>1931867</v>
+        <v>1928261</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>1837</v>
+        <v>247</v>
       </c>
       <c r="F10" s="13">
-        <v>46065.541980787035</v>
+        <v>46054.381184259255</v>
       </c>
       <c r="G10" s="12">
-        <v>75000</v>
+        <v>1076900</v>
       </c>
       <c r="H10" s="12" t="s">
-        <v>41</v>
+        <v>267</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
@@ -35456,7 +35456,7 @@
   </sheetData>
   <autoFilter ref="A1:H1" xr:uid="{AC09894E-DA90-4159-9AB3-C36FEB6A64A4}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H11">
-      <sortCondition ref="F1"/>
+      <sortCondition ref="G1"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>